<commit_message>
Calage final des 3 bonus et des spins boostés, export SDK
Bonus 1 à 59x, bonus 2 à 160x, spins boostés à 1,5x ; simulation 3M + 1,5M spins
et 100 000 tours par bonus écrite dans le classeur.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014K11WNgkEUnnGsVcri14bC
</commit_message>
<xml_diff>
--- a/modele_maths/modele_maths.xlsx
+++ b/modele_maths/modele_maths.xlsx
@@ -54,11 +54,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
-    <numFmt numFmtId="164" formatCode="0.00&quot;x&quot;"/>
-    <numFmt numFmtId="165" formatCode="0.0000"/>
-    <numFmt numFmtId="166" formatCode="0.0000%"/>
-    <numFmt numFmtId="167" formatCode="0.000%"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.00&quot;x&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0000%"/>
+    <numFmt numFmtId="168" formatCode="0.000%"/>
     <numFmt numFmtId="169" formatCode="0.000000%"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
@@ -168,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -203,10 +203,10 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="1" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -216,9 +216,9 @@
     <xf numFmtId="3" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -231,20 +231,36 @@
     <xf numFmtId="3" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="170" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -797,7 +813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -862,11 +878,27 @@
           <t>Date de la simulation</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="43" t="n"/>
-      <c r="H5" s="43" t="n"/>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 22:32</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-09 22:32</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>0 x</t>
+        </is>
+      </c>
+      <c r="G5" s="56" t="n">
+        <v>0.6996192733293443</v>
+      </c>
+      <c r="H5" s="56" t="n">
+        <v>0.7006786108775992</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -874,11 +906,23 @@
           <t>Spins simulés</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n"/>
-      <c r="C6" s="20" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="43" t="n"/>
-      <c r="H6" s="43" t="n"/>
+      <c r="B6" s="20" t="n">
+        <v>3078340</v>
+      </c>
+      <c r="C6" s="20" t="n">
+        <v>1532014</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>0 – 1 x</t>
+        </is>
+      </c>
+      <c r="G6" s="56" t="n">
+        <v>0.180270346466384</v>
+      </c>
+      <c r="H6" s="56" t="n">
+        <v>0.1776766631435479</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -886,11 +930,23 @@
           <t>Coût d'un spin (x mise)</t>
         </is>
       </c>
-      <c r="B7" s="44" t="n"/>
-      <c r="C7" s="44" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="43" t="n"/>
-      <c r="H7" s="43" t="n"/>
+      <c r="B7" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="44" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>1 – 5 x</t>
+        </is>
+      </c>
+      <c r="G7" s="56" t="n">
+        <v>0.1107845617342869</v>
+      </c>
+      <c r="H7" s="56" t="n">
+        <v>0.1076111619620006</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -898,11 +954,23 @@
           <t>RTP des spins (hors bonus)</t>
         </is>
       </c>
-      <c r="B8" s="29" t="n"/>
-      <c r="C8" s="29" t="n"/>
-      <c r="F8" s="6" t="n"/>
-      <c r="G8" s="43" t="n"/>
-      <c r="H8" s="43" t="n"/>
+      <c r="B8" s="29" t="n">
+        <v>0.5888030533550216</v>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>0.371916280648126</v>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>5 – 20 x</t>
+        </is>
+      </c>
+      <c r="G8" s="56" t="n">
+        <v>0.007767980995735308</v>
+      </c>
+      <c r="H8" s="56" t="n">
+        <v>0.01159278730710878</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
@@ -910,11 +978,23 @@
           <t>RTP des bonus</t>
         </is>
       </c>
-      <c r="B9" s="29" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="43" t="n"/>
-      <c r="H9" s="43" t="n"/>
+      <c r="B9" s="29" t="n">
+        <v>0.3568642256532524</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>0.5845663256446606</v>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>20 – 100 x</t>
+        </is>
+      </c>
+      <c r="G9" s="56" t="n">
+        <v>0.0005480605065355157</v>
+      </c>
+      <c r="H9" s="56" t="n">
+        <v>0.0008497950419780626</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
@@ -922,11 +1002,23 @@
           <t>RTP total</t>
         </is>
       </c>
-      <c r="B10" s="29" t="n"/>
-      <c r="C10" s="29" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="43" t="n"/>
-      <c r="H10" s="43" t="n"/>
+      <c r="B10" s="29" t="n">
+        <v>0.9456672790082743</v>
+      </c>
+      <c r="C10" s="29" t="n">
+        <v>0.9564826062927866</v>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>100 – 1000 x</t>
+        </is>
+      </c>
+      <c r="G10" s="56" t="n">
+        <v>0.0008623815027859917</v>
+      </c>
+      <c r="H10" s="56" t="n">
+        <v>0.001276657364401604</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
@@ -934,11 +1026,23 @@
           <t>Marge d'erreur RTP (± à 95 %)</t>
         </is>
       </c>
-      <c r="B11" s="43" t="n"/>
-      <c r="C11" s="43" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="43" t="n"/>
-      <c r="H11" s="43" t="n"/>
+      <c r="B11" s="57" t="n">
+        <v>0.0221287599106688</v>
+      </c>
+      <c r="C11" s="57" t="n">
+        <v>0.03274423528656293</v>
+      </c>
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>1000 x – max win</t>
+        </is>
+      </c>
+      <c r="G11" s="56" t="n">
+        <v>0.0001473750433704121</v>
+      </c>
+      <c r="H11" s="56" t="n">
+        <v>0.0003142633685055289</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
@@ -946,11 +1050,23 @@
           <t>Hit frequency</t>
         </is>
       </c>
-      <c r="B12" s="29" t="n"/>
-      <c r="C12" s="29" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="43" t="n"/>
-      <c r="H12" s="43" t="n"/>
+      <c r="B12" s="29" t="n">
+        <v>0.3003807266706552</v>
+      </c>
+      <c r="C12" s="29" t="n">
+        <v>0.2993213891224005</v>
+      </c>
+      <c r="F12" s="6" t="inlineStr">
+        <is>
+          <t>Max win atteint</t>
+        </is>
+      </c>
+      <c r="G12" s="56" t="n">
+        <v>2.042155708400434e-08</v>
+      </c>
+      <c r="H12" s="56" t="n">
+        <v>6.093485803643417e-08</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
@@ -958,11 +1074,15 @@
           <t>Écart-type par tour (x mise)</t>
         </is>
       </c>
-      <c r="B13" s="44" t="n"/>
-      <c r="C13" s="44" t="n"/>
+      <c r="B13" s="44" t="n">
+        <v>24.62485937985256</v>
+      </c>
+      <c r="C13" s="44" t="n">
+        <v>35.56933001456112</v>
+      </c>
       <c r="F13" s="6" t="n"/>
-      <c r="G13" s="43" t="n"/>
-      <c r="H13" s="43" t="n"/>
+      <c r="G13" s="57" t="n"/>
+      <c r="H13" s="57" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -970,11 +1090,15 @@
           <t>Bonus (tous) : 1 spin sur</t>
         </is>
       </c>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="20" t="n"/>
+      <c r="B14" s="20" t="n">
+        <v>180.8611204466233</v>
+      </c>
+      <c r="C14" s="20" t="n">
+        <v>82.76905512847853</v>
+      </c>
       <c r="F14" s="6" t="n"/>
-      <c r="G14" s="43" t="n"/>
-      <c r="H14" s="43" t="n"/>
+      <c r="G14" s="57" t="n"/>
+      <c r="H14" s="57" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
@@ -982,8 +1106,12 @@
           <t>Bonus 1 : 1 spin sur</t>
         </is>
       </c>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
+      <c r="B15" s="20" t="n">
+        <v>191.617590769405</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>89.35743087087256</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
@@ -991,8 +1119,12 @@
           <t>Bonus 2 : 1 spin sur</t>
         </is>
       </c>
-      <c r="B16" s="20" t="n"/>
-      <c r="C16" s="20" t="n"/>
+      <c r="B16" s="20" t="n">
+        <v>3344.713124725586</v>
+      </c>
+      <c r="C16" s="20" t="n">
+        <v>1182.807573562243</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
@@ -1000,8 +1132,12 @@
           <t>Bonus 3 : 1 spin sur</t>
         </is>
       </c>
-      <c r="B17" s="20" t="n"/>
-      <c r="C17" s="20" t="n"/>
+      <c r="B17" s="20" t="n">
+        <v>87738.89687603264</v>
+      </c>
+      <c r="C17" s="20" t="n">
+        <v>22049.31854210523</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
@@ -1009,8 +1145,12 @@
           <t>Bonus 1 : gain moyen (x mise)</t>
         </is>
       </c>
-      <c r="B18" s="25" t="n"/>
-      <c r="C18" s="25" t="n"/>
+      <c r="B18" s="51" t="n">
+        <v>56.03337221951441</v>
+      </c>
+      <c r="C18" s="51" t="n">
+        <v>60.66633288506777</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
@@ -1018,8 +1158,12 @@
           <t>Bonus 2 : gain moyen (x mise)</t>
         </is>
       </c>
-      <c r="B19" s="25" t="n"/>
-      <c r="C19" s="25" t="n"/>
+      <c r="B19" s="51" t="n">
+        <v>151.4935473851667</v>
+      </c>
+      <c r="C19" s="51" t="n">
+        <v>144.9355597016774</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
@@ -1027,8 +1171,12 @@
           <t>Bonus 3 : gain moyen (x mise)</t>
         </is>
       </c>
-      <c r="B20" s="25" t="n"/>
-      <c r="C20" s="25" t="n"/>
+      <c r="B20" s="51" t="n">
+        <v>1680.014489336063</v>
+      </c>
+      <c r="C20" s="51" t="n">
+        <v>1662.445562038904</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
@@ -1036,8 +1184,12 @@
           <t>Bonus 1 : FS joués en moyenne</t>
         </is>
       </c>
-      <c r="B21" s="44" t="n"/>
-      <c r="C21" s="44" t="n"/>
+      <c r="B21" s="44" t="n">
+        <v>25.93482716889917</v>
+      </c>
+      <c r="C21" s="44" t="n">
+        <v>25.8400013258818</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -1045,8 +1197,12 @@
           <t>Bonus 2 : FS joués en moyenne</t>
         </is>
       </c>
-      <c r="B22" s="44" t="n"/>
-      <c r="C22" s="44" t="n"/>
+      <c r="B22" s="44" t="n">
+        <v>30.79813034088118</v>
+      </c>
+      <c r="C22" s="44" t="n">
+        <v>31.06264515918089</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
@@ -1054,8 +1210,12 @@
           <t>Bonus 3 : FS joués en moyenne</t>
         </is>
       </c>
-      <c r="B23" s="44" t="n"/>
-      <c r="C23" s="44" t="n"/>
+      <c r="B23" s="44" t="n">
+        <v>7.049432521777755</v>
+      </c>
+      <c r="C23" s="44" t="n">
+        <v>6.837250932294474</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
@@ -1063,8 +1223,12 @@
           <t>Max win observé (x mise)</t>
         </is>
       </c>
-      <c r="B24" s="25" t="n"/>
-      <c r="C24" s="25" t="n"/>
+      <c r="B24" s="51" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C24" s="51" t="n">
+        <v>10000</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
@@ -1072,8 +1236,12 @@
           <t>Spins avec au moins 1 globe</t>
         </is>
       </c>
-      <c r="B25" s="29" t="n"/>
-      <c r="C25" s="29" t="n"/>
+      <c r="B25" s="29" t="n">
+        <v>0.0008836304957335275</v>
+      </c>
+      <c r="C25" s="29" t="n">
+        <v>0.0008619543919122412</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
@@ -1081,8 +1249,12 @@
           <t>3 étoiles : etl40b (limite 0,9)</t>
         </is>
       </c>
-      <c r="B26" s="45" t="n"/>
-      <c r="C26" s="45" t="n"/>
+      <c r="B26" s="58" t="n">
+        <v>0.5812887374764568</v>
+      </c>
+      <c r="C26" s="58" t="n">
+        <v>1.026708547209999</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
@@ -1090,8 +1262,12 @@
           <t>3 étoiles : etl10k (limite 0,8)</t>
         </is>
       </c>
-      <c r="B27" s="45" t="n"/>
-      <c r="C27" s="45" t="n"/>
+      <c r="B27" s="58" t="n">
+        <v>0.0002042155708400434</v>
+      </c>
+      <c r="C27" s="58" t="n">
+        <v>0.0006093485803643417</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
@@ -1099,53 +1275,129 @@
           <t>Max win atteint : 1 tour sur</t>
         </is>
       </c>
-      <c r="B28" s="20" t="n"/>
-      <c r="C28" s="20" t="n"/>
+      <c r="B28" s="20" t="n">
+        <v>48967862.53303246</v>
+      </c>
+      <c r="C28" s="20" t="n">
+        <v>16410967.91268604</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="inlineStr"/>
-      <c r="B29" s="46" t="n"/>
-      <c r="C29" s="46" t="n"/>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 3 symboles bonus ou moins → bonus 1)</t>
+        </is>
+      </c>
+      <c r="B29" s="46" t="n">
+        <v>0.005218727549932577</v>
+      </c>
+      <c r="C29" s="46" t="n">
+        <v>0.01119101109168041</v>
+      </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr"/>
-      <c r="B30" s="46" t="n"/>
-      <c r="C30" s="46" t="n"/>
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 3 symboles bonus ou moins → bonus 2)</t>
+        </is>
+      </c>
+      <c r="B30" s="46" t="n">
+        <v>0.0001480537857394944</v>
+      </c>
+      <c r="C30" s="46" t="n">
+        <v>0.0003972701767700076</v>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="inlineStr"/>
-      <c r="B31" s="46" t="n"/>
-      <c r="C31" s="46" t="n"/>
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 3 symboles bonus ou moins → bonus 3)</t>
+        </is>
+      </c>
+      <c r="B31" s="46" t="n">
+        <v>6.646147203031276e-06</v>
+      </c>
+      <c r="C31" s="46" t="n">
+        <v>2.631653734865039e-05</v>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="inlineStr"/>
-      <c r="B32" s="46" t="n"/>
-      <c r="C32" s="46" t="n"/>
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 4 symboles bonus → bonus 1)</t>
+        </is>
+      </c>
+      <c r="B32" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C32" s="46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="inlineStr"/>
-      <c r="B33" s="46" t="n"/>
-      <c r="C33" s="46" t="n"/>
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 4 symboles bonus → bonus 2)</t>
+        </is>
+      </c>
+      <c r="B33" s="46" t="n">
+        <v>0.0001509255176293602</v>
+      </c>
+      <c r="C33" s="46" t="n">
+        <v>0.0004481758808580007</v>
+      </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="inlineStr"/>
-      <c r="B34" s="46" t="n"/>
-      <c r="C34" s="46" t="n"/>
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 4 symboles bonus → bonus 3)</t>
+        </is>
+      </c>
+      <c r="B34" s="46" t="n">
+        <v>2.236160500698488e-06</v>
+      </c>
+      <c r="C34" s="46" t="n">
+        <v>8.835554415283003e-06</v>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="inlineStr"/>
-      <c r="B35" s="46" t="n"/>
-      <c r="C35" s="46" t="n"/>
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 5 symboles bonus → bonus 1)</t>
+        </is>
+      </c>
+      <c r="B35" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C35" s="46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="inlineStr"/>
-      <c r="B36" s="46" t="n"/>
-      <c r="C36" s="46" t="n"/>
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 5 symboles bonus → bonus 2)</t>
+        </is>
+      </c>
+      <c r="B36" s="46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr"/>
-      <c r="B37" s="46" t="n"/>
-      <c r="C37" s="46" t="n"/>
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>P(départ 5 symboles bonus → bonus 3)</t>
+        </is>
+      </c>
+      <c r="B37" s="46" t="n">
+        <v>2.515145827229671e-06</v>
+      </c>
+      <c r="C37" s="46" t="n">
+        <v>1.020078379507154e-05</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -1175,9 +1427,15 @@
           <t>Sessions simulées</t>
         </is>
       </c>
-      <c r="B41" s="20" t="n"/>
-      <c r="C41" s="20" t="n"/>
-      <c r="D41" s="20" t="n"/>
+      <c r="B41" s="20" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C41" s="20" t="n">
+        <v>100000</v>
+      </c>
+      <c r="D41" s="20" t="n">
+        <v>100000</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -1185,8 +1443,12 @@
           <t>Prix d'achat (x mise)</t>
         </is>
       </c>
-      <c r="B42" s="20" t="n"/>
-      <c r="C42" s="20" t="n"/>
+      <c r="B42" s="20" t="n">
+        <v>59</v>
+      </c>
+      <c r="C42" s="20" t="n">
+        <v>160</v>
+      </c>
       <c r="D42" s="20" t="n"/>
     </row>
     <row r="43">
@@ -1195,9 +1457,15 @@
           <t>Gain moyen (x mise)</t>
         </is>
       </c>
-      <c r="B43" s="25" t="n"/>
-      <c r="C43" s="25" t="n"/>
-      <c r="D43" s="25" t="n"/>
+      <c r="B43" s="51" t="n">
+        <v>55.57481900000001</v>
+      </c>
+      <c r="C43" s="51" t="n">
+        <v>154.061631</v>
+      </c>
+      <c r="D43" s="51" t="n">
+        <v>1697.936527</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
@@ -1205,8 +1473,12 @@
           <t>RTP au prix actuel</t>
         </is>
       </c>
-      <c r="B44" s="29" t="n"/>
-      <c r="C44" s="29" t="n"/>
+      <c r="B44" s="29" t="n">
+        <v>0.9419460847457629</v>
+      </c>
+      <c r="C44" s="29" t="n">
+        <v>0.9628851937500003</v>
+      </c>
       <c r="D44" s="29" t="n"/>
     </row>
     <row r="45">
@@ -1215,9 +1487,15 @@
           <t>Prix conseillé (gain moyen / RTP cible)</t>
         </is>
       </c>
-      <c r="B45" s="47" t="n"/>
-      <c r="C45" s="47" t="n"/>
-      <c r="D45" s="47" t="n"/>
+      <c r="B45" s="47" t="n">
+        <v>57.89043645833334</v>
+      </c>
+      <c r="C45" s="47" t="n">
+        <v>160.480865625</v>
+      </c>
+      <c r="D45" s="47" t="n">
+        <v>1768.683882291667</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
@@ -1225,9 +1503,15 @@
           <t>Gain médian (x mise)</t>
         </is>
       </c>
-      <c r="B46" s="25" t="n"/>
-      <c r="C46" s="25" t="n"/>
-      <c r="D46" s="25" t="n"/>
+      <c r="B46" s="51" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="C46" s="51" t="n">
+        <v>10</v>
+      </c>
+      <c r="D46" s="51" t="n">
+        <v>1594.7</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
@@ -1235,9 +1519,15 @@
           <t>Max win observé (x mise)</t>
         </is>
       </c>
-      <c r="B47" s="25" t="n"/>
-      <c r="C47" s="25" t="n"/>
-      <c r="D47" s="25" t="n"/>
+      <c r="B47" s="51" t="n">
+        <v>10000</v>
+      </c>
+      <c r="C47" s="51" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D47" s="51" t="n">
+        <v>7863.400000000001</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
@@ -1245,9 +1535,13 @@
           <t>3 étoiles : etl40b (limite 0,9)</t>
         </is>
       </c>
-      <c r="B48" s="45" t="n"/>
-      <c r="C48" s="45" t="n"/>
-      <c r="D48" s="45" t="n"/>
+      <c r="B48" s="58" t="n">
+        <v>5.375398000000001</v>
+      </c>
+      <c r="C48" s="58" t="n">
+        <v>4.790161999999999</v>
+      </c>
+      <c r="D48" s="58" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
@@ -1255,9 +1549,13 @@
           <t>3 étoiles : etl10k (limite 0,8)</t>
         </is>
       </c>
-      <c r="B49" s="45" t="n"/>
-      <c r="C49" s="45" t="n"/>
-      <c r="D49" s="45" t="n"/>
+      <c r="B49" s="58" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C49" s="58" t="n">
+        <v>1</v>
+      </c>
+      <c r="D49" s="58" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="12" t="inlineStr">
@@ -1286,6 +1584,132 @@
         <is>
           <t>Bonus</t>
         </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Premium 1</t>
+        </is>
+      </c>
+      <c r="C53" s="59" t="n">
+        <v>0.02966690726466617</v>
+      </c>
+      <c r="D53" s="59" t="n">
+        <v>0.03432391431590976</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>H2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Premium 2</t>
+        </is>
+      </c>
+      <c r="C54" s="59" t="n">
+        <v>0.03046711913212879</v>
+      </c>
+      <c r="D54" s="59" t="n">
+        <v>0.03661636993259879</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>H3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Premium 3</t>
+        </is>
+      </c>
+      <c r="C55" s="59" t="n">
+        <v>0.03260964870960426</v>
+      </c>
+      <c r="D55" s="59" t="n">
+        <v>0.03496682427720412</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Moyen 1</t>
+        </is>
+      </c>
+      <c r="C56" s="59" t="n">
+        <v>0.0500157887308379</v>
+      </c>
+      <c r="D56" s="59" t="n">
+        <v>0.04261317401530737</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>L1</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bas 1</t>
+        </is>
+      </c>
+      <c r="C57" s="59" t="n">
+        <v>0.1254984766173322</v>
+      </c>
+      <c r="D57" s="59" t="n">
+        <v>0.0669502752248344</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>L2</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Bas 2</t>
+        </is>
+      </c>
+      <c r="C58" s="59" t="n">
+        <v>0.1483918360915255</v>
+      </c>
+      <c r="D58" s="59" t="n">
+        <v>0.06903050605968859</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>L3</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Bas 3</t>
+        </is>
+      </c>
+      <c r="C59" s="59" t="n">
+        <v>0.1721532768089355</v>
+      </c>
+      <c r="D59" s="59" t="n">
+        <v>0.07242697255659092</v>
       </c>
     </row>
   </sheetData>
@@ -1766,11 +2190,11 @@
           <t>3 étoiles : etl40b (limite 0,9)</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="48">
         <f>Simulation!B26</f>
         <v/>
       </c>
-      <c r="C30" s="16">
+      <c r="C30" s="48">
         <f>Simulation!C26</f>
         <v/>
       </c>
@@ -1786,11 +2210,11 @@
           <t>3 étoiles : etl10k (limite 0,8)</t>
         </is>
       </c>
-      <c r="B31" s="16">
+      <c r="B31" s="48">
         <f>Simulation!B27</f>
         <v/>
       </c>
-      <c r="C31" s="16">
+      <c r="C31" s="48">
         <f>Simulation!C27</f>
         <v/>
       </c>
@@ -1806,11 +2230,11 @@
           <t>Max win observé (x mise)</t>
         </is>
       </c>
-      <c r="B32" s="17">
+      <c r="B32" s="49">
         <f>Simulation!B24</f>
         <v/>
       </c>
-      <c r="C32" s="17">
+      <c r="C32" s="49">
         <f>Simulation!C24</f>
         <v/>
       </c>
@@ -1959,6 +2383,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -2125,7 +2550,7 @@
           <t>Multi porté par le globe</t>
         </is>
       </c>
-      <c r="B14" s="23" t="n">
+      <c r="B14" s="50" t="n">
         <v>1</v>
       </c>
       <c r="C14" s="8" t="inlineStr">
@@ -2224,6 +2649,8 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>
@@ -2281,7 +2708,7 @@
         </is>
       </c>
       <c r="E25" s="19" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
@@ -2453,13 +2880,13 @@
           <t>PAY</t>
         </is>
       </c>
-      <c r="D4" s="23" t="n">
+      <c r="D4" s="50" t="n">
         <v>1.5</v>
       </c>
-      <c r="E4" s="23" t="n">
+      <c r="E4" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="23" t="n">
+      <c r="F4" s="50" t="n">
         <v>16</v>
       </c>
       <c r="G4" s="4" t="inlineStr"/>
@@ -2480,13 +2907,13 @@
           <t>PAY</t>
         </is>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="50" t="n">
         <v>3.5</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="50" t="n">
         <v>8</v>
       </c>
       <c r="G5" s="4" t="inlineStr"/>
@@ -2507,13 +2934,13 @@
           <t>PAY</t>
         </is>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="50" t="n">
         <v>0.8</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="50" t="n">
         <v>2.2</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="50" t="n">
         <v>5.5</v>
       </c>
       <c r="G6" s="4" t="inlineStr"/>
@@ -2534,13 +2961,13 @@
           <t>PAY</t>
         </is>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="50" t="n">
         <v>0.6</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="50" t="n">
         <v>1.4</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="50" t="n">
         <v>3.4</v>
       </c>
       <c r="G7" s="4" t="inlineStr"/>
@@ -2561,13 +2988,13 @@
           <t>PAY</t>
         </is>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="50" t="n">
         <v>0.3</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="50" t="n">
         <v>0.8</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="50" t="n">
         <v>2.2</v>
       </c>
       <c r="G8" s="4" t="inlineStr"/>
@@ -2588,13 +3015,13 @@
           <t>PAY</t>
         </is>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="50" t="n">
         <v>0.25</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="50" t="n">
         <v>0.7</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="50" t="n">
         <v>1.7</v>
       </c>
       <c r="G9" s="4" t="inlineStr"/>
@@ -2615,13 +3042,13 @@
           <t>PAY</t>
         </is>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="50" t="n">
         <v>0.2</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="50" t="n">
         <v>0.6</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="50" t="n">
         <v>1.4</v>
       </c>
       <c r="G10" s="4" t="inlineStr"/>
@@ -2642,13 +3069,13 @@
           <t>SCATTER</t>
         </is>
       </c>
-      <c r="D11" s="25" t="n">
+      <c r="D11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="25" t="n">
+      <c r="E11" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="25" t="n">
+      <c r="F11" s="51" t="n">
         <v>0</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
@@ -2673,13 +3100,13 @@
           <t>GLOBE</t>
         </is>
       </c>
-      <c r="D12" s="25" t="n">
+      <c r="D12" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="25" t="n">
+      <c r="E12" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="25" t="n">
+      <c r="F12" s="51" t="n">
         <v>0</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -2784,28 +3211,28 @@
         <f>B4</f>
         <v/>
       </c>
-      <c r="C18" s="23" t="n">
+      <c r="C18" s="50" t="n">
         <v>2.5</v>
       </c>
-      <c r="D18" s="23" t="n">
+      <c r="D18" s="50" t="n">
         <v>3.5</v>
       </c>
-      <c r="E18" s="23" t="n">
+      <c r="E18" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="F18" s="23" t="n">
+      <c r="F18" s="50" t="n">
         <v>7</v>
       </c>
-      <c r="G18" s="23" t="n">
+      <c r="G18" s="50" t="n">
         <v>12</v>
       </c>
-      <c r="H18" s="23" t="n">
+      <c r="H18" s="50" t="n">
         <v>25</v>
       </c>
-      <c r="I18" s="23" t="n">
+      <c r="I18" s="50" t="n">
         <v>60</v>
       </c>
-      <c r="J18" s="23" t="n">
+      <c r="J18" s="50" t="n">
         <v>180</v>
       </c>
     </row>
@@ -2818,28 +3245,28 @@
         <f>B5</f>
         <v/>
       </c>
-      <c r="C19" s="23" t="n">
+      <c r="C19" s="50" t="n">
         <v>1.8</v>
       </c>
-      <c r="D19" s="23" t="n">
+      <c r="D19" s="50" t="n">
         <v>2.5</v>
       </c>
-      <c r="E19" s="23" t="n">
+      <c r="E19" s="50" t="n">
         <v>3.5</v>
       </c>
-      <c r="F19" s="23" t="n">
+      <c r="F19" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="G19" s="23" t="n">
+      <c r="G19" s="50" t="n">
         <v>8</v>
       </c>
-      <c r="H19" s="23" t="n">
+      <c r="H19" s="50" t="n">
         <v>18</v>
       </c>
-      <c r="I19" s="23" t="n">
+      <c r="I19" s="50" t="n">
         <v>40</v>
       </c>
-      <c r="J19" s="23" t="n">
+      <c r="J19" s="50" t="n">
         <v>120</v>
       </c>
     </row>
@@ -2852,28 +3279,28 @@
         <f>B6</f>
         <v/>
       </c>
-      <c r="C20" s="23" t="n">
+      <c r="C20" s="50" t="n">
         <v>1.2</v>
       </c>
-      <c r="D20" s="23" t="n">
+      <c r="D20" s="50" t="n">
         <v>1.8</v>
       </c>
-      <c r="E20" s="23" t="n">
+      <c r="E20" s="50" t="n">
         <v>2.5</v>
       </c>
-      <c r="F20" s="23" t="n">
+      <c r="F20" s="50" t="n">
         <v>3.5</v>
       </c>
-      <c r="G20" s="23" t="n">
+      <c r="G20" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="H20" s="23" t="n">
+      <c r="H20" s="50" t="n">
         <v>12</v>
       </c>
-      <c r="I20" s="23" t="n">
+      <c r="I20" s="50" t="n">
         <v>30</v>
       </c>
-      <c r="J20" s="23" t="n">
+      <c r="J20" s="50" t="n">
         <v>90</v>
       </c>
     </row>
@@ -2886,28 +3313,28 @@
         <f>B7</f>
         <v/>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C21" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="50" t="n">
         <v>1.2</v>
       </c>
-      <c r="E21" s="23" t="n">
+      <c r="E21" s="50" t="n">
         <v>1.8</v>
       </c>
-      <c r="F21" s="23" t="n">
+      <c r="F21" s="50" t="n">
         <v>2.5</v>
       </c>
-      <c r="G21" s="23" t="n">
+      <c r="G21" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="H21" s="23" t="n">
+      <c r="H21" s="50" t="n">
         <v>10</v>
       </c>
-      <c r="I21" s="23" t="n">
+      <c r="I21" s="50" t="n">
         <v>25</v>
       </c>
-      <c r="J21" s="23" t="n">
+      <c r="J21" s="50" t="n">
         <v>60</v>
       </c>
     </row>
@@ -2920,28 +3347,28 @@
         <f>B8</f>
         <v/>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C22" s="50" t="n">
         <v>0.6</v>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="50" t="n">
         <v>0.8</v>
       </c>
-      <c r="E22" s="23" t="n">
+      <c r="E22" s="50" t="n">
         <v>1.2</v>
       </c>
-      <c r="F22" s="23" t="n">
+      <c r="F22" s="50" t="n">
         <v>1.8</v>
       </c>
-      <c r="G22" s="23" t="n">
+      <c r="G22" s="50" t="n">
         <v>3.5</v>
       </c>
-      <c r="H22" s="23" t="n">
+      <c r="H22" s="50" t="n">
         <v>7</v>
       </c>
-      <c r="I22" s="23" t="n">
+      <c r="I22" s="50" t="n">
         <v>18</v>
       </c>
-      <c r="J22" s="23" t="n">
+      <c r="J22" s="50" t="n">
         <v>50</v>
       </c>
     </row>
@@ -2954,28 +3381,28 @@
         <f>B9</f>
         <v/>
       </c>
-      <c r="C23" s="23" t="n">
+      <c r="C23" s="50" t="n">
         <v>0.5</v>
       </c>
-      <c r="D23" s="23" t="n">
+      <c r="D23" s="50" t="n">
         <v>0.7</v>
       </c>
-      <c r="E23" s="23" t="n">
+      <c r="E23" s="50" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="23" t="n">
+      <c r="F23" s="50" t="n">
         <v>1.5</v>
       </c>
-      <c r="G23" s="23" t="n">
+      <c r="G23" s="50" t="n">
         <v>3</v>
       </c>
-      <c r="H23" s="23" t="n">
+      <c r="H23" s="50" t="n">
         <v>6</v>
       </c>
-      <c r="I23" s="23" t="n">
+      <c r="I23" s="50" t="n">
         <v>15</v>
       </c>
-      <c r="J23" s="23" t="n">
+      <c r="J23" s="50" t="n">
         <v>35</v>
       </c>
     </row>
@@ -2988,28 +3415,28 @@
         <f>B10</f>
         <v/>
       </c>
-      <c r="C24" s="23" t="n">
+      <c r="C24" s="50" t="n">
         <v>0.4</v>
       </c>
-      <c r="D24" s="23" t="n">
+      <c r="D24" s="50" t="n">
         <v>0.6</v>
       </c>
-      <c r="E24" s="23" t="n">
+      <c r="E24" s="50" t="n">
         <v>0.8</v>
       </c>
-      <c r="F24" s="23" t="n">
+      <c r="F24" s="50" t="n">
         <v>1.2</v>
       </c>
-      <c r="G24" s="23" t="n">
+      <c r="G24" s="50" t="n">
         <v>2.5</v>
       </c>
-      <c r="H24" s="23" t="n">
+      <c r="H24" s="50" t="n">
         <v>5</v>
       </c>
-      <c r="I24" s="23" t="n">
+      <c r="I24" s="50" t="n">
         <v>12</v>
       </c>
-      <c r="J24" s="23" t="n">
+      <c r="J24" s="50" t="n">
         <v>30</v>
       </c>
     </row>
@@ -3022,28 +3449,28 @@
         <f>B11</f>
         <v/>
       </c>
-      <c r="C25" s="25" t="n">
+      <c r="C25" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="25" t="n">
+      <c r="D25" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="25" t="n">
+      <c r="E25" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="25" t="n">
+      <c r="F25" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="25" t="n">
+      <c r="G25" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="25" t="n">
+      <c r="H25" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I25" s="25" t="n">
+      <c r="I25" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="J25" s="25" t="n">
+      <c r="J25" s="51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3056,28 +3483,28 @@
         <f>B12</f>
         <v/>
       </c>
-      <c r="C26" s="25" t="n">
+      <c r="C26" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="25" t="n">
+      <c r="D26" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="25" t="n">
+      <c r="E26" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="25" t="n">
+      <c r="F26" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="G26" s="25" t="n">
+      <c r="G26" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="H26" s="25" t="n">
+      <c r="H26" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="I26" s="25" t="n">
+      <c r="I26" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="J26" s="25" t="n">
+      <c r="J26" s="51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -6808,7 +7235,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="n">
+      <c r="A5" s="50" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="19" t="n">
@@ -6841,7 +7268,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="n">
+      <c r="A6" s="50" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="19" t="n">
@@ -6874,7 +7301,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="n">
+      <c r="A7" s="50" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="19" t="n">
@@ -6907,7 +7334,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="n">
+      <c r="A8" s="50" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="19" t="n">
@@ -6940,7 +7367,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="n">
+      <c r="A9" s="50" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="19" t="n">
@@ -6973,7 +7400,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="n">
+      <c r="A10" s="50" t="n">
         <v>10</v>
       </c>
       <c r="B10" s="19" t="n">
@@ -7006,7 +7433,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="n">
+      <c r="A11" s="50" t="n">
         <v>20</v>
       </c>
       <c r="B11" s="19" t="n">
@@ -7039,7 +7466,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="n">
+      <c r="A12" s="50" t="n">
         <v>50</v>
       </c>
       <c r="B12" s="19" t="n">
@@ -7072,7 +7499,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="n">
+      <c r="A13" s="50" t="n">
         <v>100</v>
       </c>
       <c r="B13" s="19" t="n">
@@ -7153,19 +7580,19 @@
       <c r="C15" s="33" t="inlineStr"/>
       <c r="D15" s="33" t="inlineStr"/>
       <c r="E15" s="33" t="inlineStr"/>
-      <c r="F15" s="34">
+      <c r="F15" s="52">
         <f>SUMPRODUCT($A$5:$A$13,F5:F13)</f>
         <v/>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="52">
         <f>SUMPRODUCT($A$5:$A$13,G5:G13)</f>
         <v/>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="52">
         <f>SUMPRODUCT($A$5:$A$13,H5:H13)</f>
         <v/>
       </c>
-      <c r="I15" s="34">
+      <c r="I15" s="52">
         <f>SUMPRODUCT($A$5:$A$13,I5:I13)</f>
         <v/>
       </c>
@@ -7317,15 +7744,15 @@
         <f>Poids!M5</f>
         <v/>
       </c>
-      <c r="H5" s="36">
+      <c r="H5" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C5*D5*E5*((1-NB_LIGNES*Poids!$L$12)*(1-F5/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F5/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C5*D5*E5*(1-F5))</f>
         <v/>
       </c>
-      <c r="I5" s="36">
+      <c r="I5" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C5*D5*E5*F5*((1-NB_LIGNES*Poids!$M$12)*(1-G5/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G5/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C5*D5*E5*F5*(1-G5))</f>
         <v/>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C5*D5*E5*F5*G5</f>
         <v/>
       </c>
@@ -7367,15 +7794,15 @@
         <f>Poids!M6</f>
         <v/>
       </c>
-      <c r="H6" s="36">
+      <c r="H6" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C6*D6*E6*((1-NB_LIGNES*Poids!$L$12)*(1-F6/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F6/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C6*D6*E6*(1-F6))</f>
         <v/>
       </c>
-      <c r="I6" s="36">
+      <c r="I6" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C6*D6*E6*F6*((1-NB_LIGNES*Poids!$M$12)*(1-G6/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G6/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C6*D6*E6*F6*(1-G6))</f>
         <v/>
       </c>
-      <c r="J6" s="36">
+      <c r="J6" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C6*D6*E6*F6*G6</f>
         <v/>
       </c>
@@ -7417,15 +7844,15 @@
         <f>Poids!M7</f>
         <v/>
       </c>
-      <c r="H7" s="36">
+      <c r="H7" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C7*D7*E7*((1-NB_LIGNES*Poids!$L$12)*(1-F7/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F7/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C7*D7*E7*(1-F7))</f>
         <v/>
       </c>
-      <c r="I7" s="36">
+      <c r="I7" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C7*D7*E7*F7*((1-NB_LIGNES*Poids!$M$12)*(1-G7/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G7/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C7*D7*E7*F7*(1-G7))</f>
         <v/>
       </c>
-      <c r="J7" s="36">
+      <c r="J7" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C7*D7*E7*F7*G7</f>
         <v/>
       </c>
@@ -7467,15 +7894,15 @@
         <f>Poids!M8</f>
         <v/>
       </c>
-      <c r="H8" s="36">
+      <c r="H8" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C8*D8*E8*((1-NB_LIGNES*Poids!$L$12)*(1-F8/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F8/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C8*D8*E8*(1-F8))</f>
         <v/>
       </c>
-      <c r="I8" s="36">
+      <c r="I8" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C8*D8*E8*F8*((1-NB_LIGNES*Poids!$M$12)*(1-G8/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G8/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C8*D8*E8*F8*(1-G8))</f>
         <v/>
       </c>
-      <c r="J8" s="36">
+      <c r="J8" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C8*D8*E8*F8*G8</f>
         <v/>
       </c>
@@ -7517,15 +7944,15 @@
         <f>Poids!M9</f>
         <v/>
       </c>
-      <c r="H9" s="36">
+      <c r="H9" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C9*D9*E9*((1-NB_LIGNES*Poids!$L$12)*(1-F9/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F9/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C9*D9*E9*(1-F9))</f>
         <v/>
       </c>
-      <c r="I9" s="36">
+      <c r="I9" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C9*D9*E9*F9*((1-NB_LIGNES*Poids!$M$12)*(1-G9/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G9/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C9*D9*E9*F9*(1-G9))</f>
         <v/>
       </c>
-      <c r="J9" s="36">
+      <c r="J9" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C9*D9*E9*F9*G9</f>
         <v/>
       </c>
@@ -7567,15 +7994,15 @@
         <f>Poids!M10</f>
         <v/>
       </c>
-      <c r="H10" s="36">
+      <c r="H10" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C10*D10*E10*((1-NB_LIGNES*Poids!$L$12)*(1-F10/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F10/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C10*D10*E10*(1-F10))</f>
         <v/>
       </c>
-      <c r="I10" s="36">
+      <c r="I10" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C10*D10*E10*F10*((1-NB_LIGNES*Poids!$M$12)*(1-G10/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G10/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C10*D10*E10*F10*(1-G10))</f>
         <v/>
       </c>
-      <c r="J10" s="36">
+      <c r="J10" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C10*D10*E10*F10*G10</f>
         <v/>
       </c>
@@ -7617,15 +8044,15 @@
         <f>Poids!M11</f>
         <v/>
       </c>
-      <c r="H11" s="36">
+      <c r="H11" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C11*D11*E11*((1-NB_LIGNES*Poids!$L$12)*(1-F11/(1-Poids!$L$12))^NB_LIGNES+NB_LIGNES*Poids!$L$12*(1-F11/(1-Poids!$L$12))^(NB_LIGNES-1)),NB_PAYLINES*C11*D11*E11*(1-F11))</f>
         <v/>
       </c>
-      <c r="I11" s="36">
+      <c r="I11" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C11*D11*E11*F11*((1-NB_LIGNES*Poids!$M$12)*(1-G11/(1-Poids!$M$12))^NB_LIGNES+NB_LIGNES*Poids!$M$12*(1-G11/(1-Poids!$M$12))^(NB_LIGNES-1)),NB_PAYLINES*C11*D11*E11*F11*(1-G11))</f>
         <v/>
       </c>
-      <c r="J11" s="36">
+      <c r="J11" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C11*D11*E11*F11*G11</f>
         <v/>
       </c>
@@ -7649,15 +8076,15 @@
       <c r="E12" s="33" t="inlineStr"/>
       <c r="F12" s="33" t="inlineStr"/>
       <c r="G12" s="33" t="inlineStr"/>
-      <c r="H12" s="37">
+      <c r="H12" s="54">
         <f>SUM(H5:H11)</f>
         <v/>
       </c>
-      <c r="I12" s="37">
+      <c r="I12" s="54">
         <f>SUM(I5:I11)</f>
         <v/>
       </c>
-      <c r="J12" s="37">
+      <c r="J12" s="54">
         <f>SUM(J5:J11)</f>
         <v/>
       </c>
@@ -7768,15 +8195,15 @@
         <f>Poids!M33</f>
         <v/>
       </c>
-      <c r="H17" s="36">
+      <c r="H17" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C17*D17*E17*((1-NB_LIGNES*Poids!$L$40)*(1-F17/(1-Poids!$L$40))^NB_LIGNES+NB_LIGNES*Poids!$L$40*(1-F17/(1-Poids!$L$40))^(NB_LIGNES-1)),NB_PAYLINES*C17*D17*E17*(1-F17))</f>
         <v/>
       </c>
-      <c r="I17" s="36">
+      <c r="I17" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C17*D17*E17*F17*((1-NB_LIGNES*Poids!$M$40)*(1-G17/(1-Poids!$M$40))^NB_LIGNES+NB_LIGNES*Poids!$M$40*(1-G17/(1-Poids!$M$40))^(NB_LIGNES-1)),NB_PAYLINES*C17*D17*E17*F17*(1-G17))</f>
         <v/>
       </c>
-      <c r="J17" s="36">
+      <c r="J17" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C17*D17*E17*F17*G17</f>
         <v/>
       </c>
@@ -7818,15 +8245,15 @@
         <f>Poids!M34</f>
         <v/>
       </c>
-      <c r="H18" s="36">
+      <c r="H18" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C18*D18*E18*((1-NB_LIGNES*Poids!$L$40)*(1-F18/(1-Poids!$L$40))^NB_LIGNES+NB_LIGNES*Poids!$L$40*(1-F18/(1-Poids!$L$40))^(NB_LIGNES-1)),NB_PAYLINES*C18*D18*E18*(1-F18))</f>
         <v/>
       </c>
-      <c r="I18" s="36">
+      <c r="I18" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C18*D18*E18*F18*((1-NB_LIGNES*Poids!$M$40)*(1-G18/(1-Poids!$M$40))^NB_LIGNES+NB_LIGNES*Poids!$M$40*(1-G18/(1-Poids!$M$40))^(NB_LIGNES-1)),NB_PAYLINES*C18*D18*E18*F18*(1-G18))</f>
         <v/>
       </c>
-      <c r="J18" s="36">
+      <c r="J18" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C18*D18*E18*F18*G18</f>
         <v/>
       </c>
@@ -7868,15 +8295,15 @@
         <f>Poids!M35</f>
         <v/>
       </c>
-      <c r="H19" s="36">
+      <c r="H19" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C19*D19*E19*((1-NB_LIGNES*Poids!$L$40)*(1-F19/(1-Poids!$L$40))^NB_LIGNES+NB_LIGNES*Poids!$L$40*(1-F19/(1-Poids!$L$40))^(NB_LIGNES-1)),NB_PAYLINES*C19*D19*E19*(1-F19))</f>
         <v/>
       </c>
-      <c r="I19" s="36">
+      <c r="I19" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C19*D19*E19*F19*((1-NB_LIGNES*Poids!$M$40)*(1-G19/(1-Poids!$M$40))^NB_LIGNES+NB_LIGNES*Poids!$M$40*(1-G19/(1-Poids!$M$40))^(NB_LIGNES-1)),NB_PAYLINES*C19*D19*E19*F19*(1-G19))</f>
         <v/>
       </c>
-      <c r="J19" s="36">
+      <c r="J19" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C19*D19*E19*F19*G19</f>
         <v/>
       </c>
@@ -7918,15 +8345,15 @@
         <f>Poids!M36</f>
         <v/>
       </c>
-      <c r="H20" s="36">
+      <c r="H20" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C20*D20*E20*((1-NB_LIGNES*Poids!$L$40)*(1-F20/(1-Poids!$L$40))^NB_LIGNES+NB_LIGNES*Poids!$L$40*(1-F20/(1-Poids!$L$40))^(NB_LIGNES-1)),NB_PAYLINES*C20*D20*E20*(1-F20))</f>
         <v/>
       </c>
-      <c r="I20" s="36">
+      <c r="I20" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C20*D20*E20*F20*((1-NB_LIGNES*Poids!$M$40)*(1-G20/(1-Poids!$M$40))^NB_LIGNES+NB_LIGNES*Poids!$M$40*(1-G20/(1-Poids!$M$40))^(NB_LIGNES-1)),NB_PAYLINES*C20*D20*E20*F20*(1-G20))</f>
         <v/>
       </c>
-      <c r="J20" s="36">
+      <c r="J20" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C20*D20*E20*F20*G20</f>
         <v/>
       </c>
@@ -7968,15 +8395,15 @@
         <f>Poids!M37</f>
         <v/>
       </c>
-      <c r="H21" s="36">
+      <c r="H21" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C21*D21*E21*((1-NB_LIGNES*Poids!$L$40)*(1-F21/(1-Poids!$L$40))^NB_LIGNES+NB_LIGNES*Poids!$L$40*(1-F21/(1-Poids!$L$40))^(NB_LIGNES-1)),NB_PAYLINES*C21*D21*E21*(1-F21))</f>
         <v/>
       </c>
-      <c r="I21" s="36">
+      <c r="I21" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C21*D21*E21*F21*((1-NB_LIGNES*Poids!$M$40)*(1-G21/(1-Poids!$M$40))^NB_LIGNES+NB_LIGNES*Poids!$M$40*(1-G21/(1-Poids!$M$40))^(NB_LIGNES-1)),NB_PAYLINES*C21*D21*E21*F21*(1-G21))</f>
         <v/>
       </c>
-      <c r="J21" s="36">
+      <c r="J21" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C21*D21*E21*F21*G21</f>
         <v/>
       </c>
@@ -8018,15 +8445,15 @@
         <f>Poids!M38</f>
         <v/>
       </c>
-      <c r="H22" s="36">
+      <c r="H22" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C22*D22*E22*((1-NB_LIGNES*Poids!$L$40)*(1-F22/(1-Poids!$L$40))^NB_LIGNES+NB_LIGNES*Poids!$L$40*(1-F22/(1-Poids!$L$40))^(NB_LIGNES-1)),NB_PAYLINES*C22*D22*E22*(1-F22))</f>
         <v/>
       </c>
-      <c r="I22" s="36">
+      <c r="I22" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C22*D22*E22*F22*((1-NB_LIGNES*Poids!$M$40)*(1-G22/(1-Poids!$M$40))^NB_LIGNES+NB_LIGNES*Poids!$M$40*(1-G22/(1-Poids!$M$40))^(NB_LIGNES-1)),NB_PAYLINES*C22*D22*E22*F22*(1-G22))</f>
         <v/>
       </c>
-      <c r="J22" s="36">
+      <c r="J22" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C22*D22*E22*F22*G22</f>
         <v/>
       </c>
@@ -8068,15 +8495,15 @@
         <f>Poids!M39</f>
         <v/>
       </c>
-      <c r="H23" s="36">
+      <c r="H23" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^3*C23*D23*E23*((1-NB_LIGNES*Poids!$L$40)*(1-F23/(1-Poids!$L$40))^NB_LIGNES+NB_LIGNES*Poids!$L$40*(1-F23/(1-Poids!$L$40))^(NB_LIGNES-1)),NB_PAYLINES*C23*D23*E23*(1-F23))</f>
         <v/>
       </c>
-      <c r="I23" s="36">
+      <c r="I23" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^4*C23*D23*E23*F23*((1-NB_LIGNES*Poids!$M$40)*(1-G23/(1-Poids!$M$40))^NB_LIGNES+NB_LIGNES*Poids!$M$40*(1-G23/(1-Poids!$M$40))^(NB_LIGNES-1)),NB_PAYLINES*C23*D23*E23*F23*(1-G23))</f>
         <v/>
       </c>
-      <c r="J23" s="36">
+      <c r="J23" s="53">
         <f>IF(MODE_GAIN="WAYS",NB_LIGNES^5,NB_PAYLINES)*C23*D23*E23*F23*G23</f>
         <v/>
       </c>
@@ -8100,15 +8527,15 @@
       <c r="E24" s="33" t="inlineStr"/>
       <c r="F24" s="33" t="inlineStr"/>
       <c r="G24" s="33" t="inlineStr"/>
-      <c r="H24" s="37">
+      <c r="H24" s="54">
         <f>SUM(H17:H23)</f>
         <v/>
       </c>
-      <c r="I24" s="37">
+      <c r="I24" s="54">
         <f>SUM(I17:I23)</f>
         <v/>
       </c>
-      <c r="J24" s="37">
+      <c r="J24" s="54">
         <f>SUM(J17:J23)</f>
         <v/>
       </c>
@@ -8214,23 +8641,23 @@
           <t>Symbole bonus — base</t>
         </is>
       </c>
-      <c r="B5" s="38">
+      <c r="B5" s="55">
         <f>Poids!I12</f>
         <v/>
       </c>
-      <c r="C5" s="38">
+      <c r="C5" s="55">
         <f>Poids!J12</f>
         <v/>
       </c>
-      <c r="D5" s="38">
+      <c r="D5" s="55">
         <f>Poids!K12</f>
         <v/>
       </c>
-      <c r="E5" s="38">
+      <c r="E5" s="55">
         <f>Poids!L12</f>
         <v/>
       </c>
-      <c r="F5" s="38">
+      <c r="F5" s="55">
         <f>Poids!M12</f>
         <v/>
       </c>
@@ -8241,23 +8668,23 @@
           <t>Symbole bonus — boost</t>
         </is>
       </c>
-      <c r="B6" s="38">
+      <c r="B6" s="55">
         <f>Poids!I26</f>
         <v/>
       </c>
-      <c r="C6" s="38">
+      <c r="C6" s="55">
         <f>Poids!J26</f>
         <v/>
       </c>
-      <c r="D6" s="38">
+      <c r="D6" s="55">
         <f>Poids!K26</f>
         <v/>
       </c>
-      <c r="E6" s="38">
+      <c r="E6" s="55">
         <f>Poids!L26</f>
         <v/>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="55">
         <f>Poids!M26</f>
         <v/>
       </c>
@@ -8268,23 +8695,23 @@
           <t>Symbole bonus — FS bonus 1</t>
         </is>
       </c>
-      <c r="B7" s="38">
+      <c r="B7" s="55">
         <f>Poids!I40</f>
         <v/>
       </c>
-      <c r="C7" s="38">
+      <c r="C7" s="55">
         <f>Poids!J40</f>
         <v/>
       </c>
-      <c r="D7" s="38">
+      <c r="D7" s="55">
         <f>Poids!K40</f>
         <v/>
       </c>
-      <c r="E7" s="38">
+      <c r="E7" s="55">
         <f>Poids!L40</f>
         <v/>
       </c>
-      <c r="F7" s="38">
+      <c r="F7" s="55">
         <f>Poids!M40</f>
         <v/>
       </c>
@@ -8295,23 +8722,23 @@
           <t>Symbole bonus — FS bonus 2</t>
         </is>
       </c>
-      <c r="B8" s="38">
+      <c r="B8" s="55">
         <f>Poids!I54</f>
         <v/>
       </c>
-      <c r="C8" s="38">
+      <c r="C8" s="55">
         <f>Poids!J54</f>
         <v/>
       </c>
-      <c r="D8" s="38">
+      <c r="D8" s="55">
         <f>Poids!K54</f>
         <v/>
       </c>
-      <c r="E8" s="38">
+      <c r="E8" s="55">
         <f>Poids!L54</f>
         <v/>
       </c>
-      <c r="F8" s="38">
+      <c r="F8" s="55">
         <f>Poids!M54</f>
         <v/>
       </c>
@@ -8322,23 +8749,23 @@
           <t>Symbole bonus — FS bonus 3</t>
         </is>
       </c>
-      <c r="B9" s="38">
+      <c r="B9" s="55">
         <f>Poids!I68</f>
         <v/>
       </c>
-      <c r="C9" s="38">
+      <c r="C9" s="55">
         <f>Poids!J68</f>
         <v/>
       </c>
-      <c r="D9" s="38">
+      <c r="D9" s="55">
         <f>Poids!K68</f>
         <v/>
       </c>
-      <c r="E9" s="38">
+      <c r="E9" s="55">
         <f>Poids!L68</f>
         <v/>
       </c>
-      <c r="F9" s="38">
+      <c r="F9" s="55">
         <f>Poids!M68</f>
         <v/>
       </c>
@@ -8349,23 +8776,23 @@
           <t>Globe — base</t>
         </is>
       </c>
-      <c r="B10" s="38">
+      <c r="B10" s="55">
         <f>Poids!I13</f>
         <v/>
       </c>
-      <c r="C10" s="38">
+      <c r="C10" s="55">
         <f>Poids!J13</f>
         <v/>
       </c>
-      <c r="D10" s="38">
+      <c r="D10" s="55">
         <f>Poids!K13</f>
         <v/>
       </c>
-      <c r="E10" s="38">
+      <c r="E10" s="55">
         <f>Poids!L13</f>
         <v/>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="55">
         <f>Poids!M13</f>
         <v/>
       </c>
@@ -8376,23 +8803,23 @@
           <t>Globe — boost</t>
         </is>
       </c>
-      <c r="B11" s="38">
+      <c r="B11" s="55">
         <f>Poids!I27</f>
         <v/>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="55">
         <f>Poids!J27</f>
         <v/>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="55">
         <f>Poids!K27</f>
         <v/>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="55">
         <f>Poids!L27</f>
         <v/>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="55">
         <f>Poids!M27</f>
         <v/>
       </c>
@@ -8403,23 +8830,23 @@
           <t>Globe — FS bonus 1</t>
         </is>
       </c>
-      <c r="B12" s="38">
+      <c r="B12" s="55">
         <f>Poids!I41</f>
         <v/>
       </c>
-      <c r="C12" s="38">
+      <c r="C12" s="55">
         <f>Poids!J41</f>
         <v/>
       </c>
-      <c r="D12" s="38">
+      <c r="D12" s="55">
         <f>Poids!K41</f>
         <v/>
       </c>
-      <c r="E12" s="38">
+      <c r="E12" s="55">
         <f>Poids!L41</f>
         <v/>
       </c>
-      <c r="F12" s="38">
+      <c r="F12" s="55">
         <f>Poids!M41</f>
         <v/>
       </c>
@@ -8430,23 +8857,23 @@
           <t>Globe — FS bonus 2</t>
         </is>
       </c>
-      <c r="B13" s="38">
+      <c r="B13" s="55">
         <f>Poids!I55</f>
         <v/>
       </c>
-      <c r="C13" s="38">
+      <c r="C13" s="55">
         <f>Poids!J55</f>
         <v/>
       </c>
-      <c r="D13" s="38">
+      <c r="D13" s="55">
         <f>Poids!K55</f>
         <v/>
       </c>
-      <c r="E13" s="38">
+      <c r="E13" s="55">
         <f>Poids!L55</f>
         <v/>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="55">
         <f>Poids!M55</f>
         <v/>
       </c>
@@ -8457,23 +8884,23 @@
           <t>Globe — FS bonus 3</t>
         </is>
       </c>
-      <c r="B14" s="38">
+      <c r="B14" s="55">
         <f>Poids!I69</f>
         <v/>
       </c>
-      <c r="C14" s="38">
+      <c r="C14" s="55">
         <f>Poids!J69</f>
         <v/>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="55">
         <f>Poids!K69</f>
         <v/>
       </c>
-      <c r="E14" s="38">
+      <c r="E14" s="55">
         <f>Poids!L69</f>
         <v/>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="55">
         <f>Poids!M69</f>
         <v/>
       </c>
@@ -8546,43 +8973,43 @@
       <c r="A18" s="39" t="n">
         <v>0</v>
       </c>
-      <c r="B18" s="40">
+      <c r="B18" s="56">
         <f>IF($A18=0,1-MIN(1,NB_LIGNES*B$5),IF($A18=1,MIN(1,NB_LIGNES*B$5),0))</f>
         <v/>
       </c>
-      <c r="C18" s="40">
+      <c r="C18" s="56">
         <f>B18*(1-MIN(1,NB_LIGNES*C$5))</f>
         <v/>
       </c>
-      <c r="D18" s="40">
+      <c r="D18" s="56">
         <f>C18*(1-MIN(1,NB_LIGNES*D$5))</f>
         <v/>
       </c>
-      <c r="E18" s="40">
+      <c r="E18" s="56">
         <f>D18*(1-MIN(1,NB_LIGNES*E$5))</f>
         <v/>
       </c>
-      <c r="F18" s="40">
+      <c r="F18" s="56">
         <f>E18*(1-MIN(1,NB_LIGNES*F$5))</f>
         <v/>
       </c>
-      <c r="G18" s="40">
+      <c r="G18" s="56">
         <f>IF($A18=0,1-MIN(1,NB_LIGNES*B$6),IF($A18=1,MIN(1,NB_LIGNES*B$6),0))</f>
         <v/>
       </c>
-      <c r="H18" s="40">
+      <c r="H18" s="56">
         <f>G18*(1-MIN(1,NB_LIGNES*C$6))</f>
         <v/>
       </c>
-      <c r="I18" s="40">
+      <c r="I18" s="56">
         <f>H18*(1-MIN(1,NB_LIGNES*D$6))</f>
         <v/>
       </c>
-      <c r="J18" s="40">
+      <c r="J18" s="56">
         <f>I18*(1-MIN(1,NB_LIGNES*E$6))</f>
         <v/>
       </c>
-      <c r="K18" s="40">
+      <c r="K18" s="56">
         <f>J18*(1-MIN(1,NB_LIGNES*F$6))</f>
         <v/>
       </c>
@@ -8591,43 +9018,43 @@
       <c r="A19" s="39" t="n">
         <v>1</v>
       </c>
-      <c r="B19" s="40">
+      <c r="B19" s="56">
         <f>IF($A19=0,1-MIN(1,NB_LIGNES*B$5),IF($A19=1,MIN(1,NB_LIGNES*B$5),0))</f>
         <v/>
       </c>
-      <c r="C19" s="40">
+      <c r="C19" s="56">
         <f>B19*(1-MIN(1,NB_LIGNES*C$5))+B18*MIN(1,NB_LIGNES*C$5)</f>
         <v/>
       </c>
-      <c r="D19" s="40">
+      <c r="D19" s="56">
         <f>C19*(1-MIN(1,NB_LIGNES*D$5))+C18*MIN(1,NB_LIGNES*D$5)</f>
         <v/>
       </c>
-      <c r="E19" s="40">
+      <c r="E19" s="56">
         <f>D19*(1-MIN(1,NB_LIGNES*E$5))+D18*MIN(1,NB_LIGNES*E$5)</f>
         <v/>
       </c>
-      <c r="F19" s="40">
+      <c r="F19" s="56">
         <f>E19*(1-MIN(1,NB_LIGNES*F$5))+E18*MIN(1,NB_LIGNES*F$5)</f>
         <v/>
       </c>
-      <c r="G19" s="40">
+      <c r="G19" s="56">
         <f>IF($A19=0,1-MIN(1,NB_LIGNES*B$6),IF($A19=1,MIN(1,NB_LIGNES*B$6),0))</f>
         <v/>
       </c>
-      <c r="H19" s="40">
+      <c r="H19" s="56">
         <f>G19*(1-MIN(1,NB_LIGNES*C$6))+G18*MIN(1,NB_LIGNES*C$6)</f>
         <v/>
       </c>
-      <c r="I19" s="40">
+      <c r="I19" s="56">
         <f>H19*(1-MIN(1,NB_LIGNES*D$6))+H18*MIN(1,NB_LIGNES*D$6)</f>
         <v/>
       </c>
-      <c r="J19" s="40">
+      <c r="J19" s="56">
         <f>I19*(1-MIN(1,NB_LIGNES*E$6))+I18*MIN(1,NB_LIGNES*E$6)</f>
         <v/>
       </c>
-      <c r="K19" s="40">
+      <c r="K19" s="56">
         <f>J19*(1-MIN(1,NB_LIGNES*F$6))+J18*MIN(1,NB_LIGNES*F$6)</f>
         <v/>
       </c>
@@ -8636,43 +9063,43 @@
       <c r="A20" s="39" t="n">
         <v>2</v>
       </c>
-      <c r="B20" s="40">
+      <c r="B20" s="56">
         <f>IF($A20=0,1-MIN(1,NB_LIGNES*B$5),IF($A20=1,MIN(1,NB_LIGNES*B$5),0))</f>
         <v/>
       </c>
-      <c r="C20" s="40">
+      <c r="C20" s="56">
         <f>B20*(1-MIN(1,NB_LIGNES*C$5))+B19*MIN(1,NB_LIGNES*C$5)</f>
         <v/>
       </c>
-      <c r="D20" s="40">
+      <c r="D20" s="56">
         <f>C20*(1-MIN(1,NB_LIGNES*D$5))+C19*MIN(1,NB_LIGNES*D$5)</f>
         <v/>
       </c>
-      <c r="E20" s="40">
+      <c r="E20" s="56">
         <f>D20*(1-MIN(1,NB_LIGNES*E$5))+D19*MIN(1,NB_LIGNES*E$5)</f>
         <v/>
       </c>
-      <c r="F20" s="40">
+      <c r="F20" s="56">
         <f>E20*(1-MIN(1,NB_LIGNES*F$5))+E19*MIN(1,NB_LIGNES*F$5)</f>
         <v/>
       </c>
-      <c r="G20" s="40">
+      <c r="G20" s="56">
         <f>IF($A20=0,1-MIN(1,NB_LIGNES*B$6),IF($A20=1,MIN(1,NB_LIGNES*B$6),0))</f>
         <v/>
       </c>
-      <c r="H20" s="40">
+      <c r="H20" s="56">
         <f>G20*(1-MIN(1,NB_LIGNES*C$6))+G19*MIN(1,NB_LIGNES*C$6)</f>
         <v/>
       </c>
-      <c r="I20" s="40">
+      <c r="I20" s="56">
         <f>H20*(1-MIN(1,NB_LIGNES*D$6))+H19*MIN(1,NB_LIGNES*D$6)</f>
         <v/>
       </c>
-      <c r="J20" s="40">
+      <c r="J20" s="56">
         <f>I20*(1-MIN(1,NB_LIGNES*E$6))+I19*MIN(1,NB_LIGNES*E$6)</f>
         <v/>
       </c>
-      <c r="K20" s="40">
+      <c r="K20" s="56">
         <f>J20*(1-MIN(1,NB_LIGNES*F$6))+J19*MIN(1,NB_LIGNES*F$6)</f>
         <v/>
       </c>
@@ -8681,43 +9108,43 @@
       <c r="A21" s="39" t="n">
         <v>3</v>
       </c>
-      <c r="B21" s="40">
+      <c r="B21" s="56">
         <f>IF($A21=0,1-MIN(1,NB_LIGNES*B$5),IF($A21=1,MIN(1,NB_LIGNES*B$5),0))</f>
         <v/>
       </c>
-      <c r="C21" s="40">
+      <c r="C21" s="56">
         <f>B21*(1-MIN(1,NB_LIGNES*C$5))+B20*MIN(1,NB_LIGNES*C$5)</f>
         <v/>
       </c>
-      <c r="D21" s="40">
+      <c r="D21" s="56">
         <f>C21*(1-MIN(1,NB_LIGNES*D$5))+C20*MIN(1,NB_LIGNES*D$5)</f>
         <v/>
       </c>
-      <c r="E21" s="40">
+      <c r="E21" s="56">
         <f>D21*(1-MIN(1,NB_LIGNES*E$5))+D20*MIN(1,NB_LIGNES*E$5)</f>
         <v/>
       </c>
-      <c r="F21" s="40">
+      <c r="F21" s="56">
         <f>E21*(1-MIN(1,NB_LIGNES*F$5))+E20*MIN(1,NB_LIGNES*F$5)</f>
         <v/>
       </c>
-      <c r="G21" s="40">
+      <c r="G21" s="56">
         <f>IF($A21=0,1-MIN(1,NB_LIGNES*B$6),IF($A21=1,MIN(1,NB_LIGNES*B$6),0))</f>
         <v/>
       </c>
-      <c r="H21" s="40">
+      <c r="H21" s="56">
         <f>G21*(1-MIN(1,NB_LIGNES*C$6))+G20*MIN(1,NB_LIGNES*C$6)</f>
         <v/>
       </c>
-      <c r="I21" s="40">
+      <c r="I21" s="56">
         <f>H21*(1-MIN(1,NB_LIGNES*D$6))+H20*MIN(1,NB_LIGNES*D$6)</f>
         <v/>
       </c>
-      <c r="J21" s="40">
+      <c r="J21" s="56">
         <f>I21*(1-MIN(1,NB_LIGNES*E$6))+I20*MIN(1,NB_LIGNES*E$6)</f>
         <v/>
       </c>
-      <c r="K21" s="40">
+      <c r="K21" s="56">
         <f>J21*(1-MIN(1,NB_LIGNES*F$6))+J20*MIN(1,NB_LIGNES*F$6)</f>
         <v/>
       </c>
@@ -8726,43 +9153,43 @@
       <c r="A22" s="39" t="n">
         <v>4</v>
       </c>
-      <c r="B22" s="40">
+      <c r="B22" s="56">
         <f>IF($A22=0,1-MIN(1,NB_LIGNES*B$5),IF($A22=1,MIN(1,NB_LIGNES*B$5),0))</f>
         <v/>
       </c>
-      <c r="C22" s="40">
+      <c r="C22" s="56">
         <f>B22*(1-MIN(1,NB_LIGNES*C$5))+B21*MIN(1,NB_LIGNES*C$5)</f>
         <v/>
       </c>
-      <c r="D22" s="40">
+      <c r="D22" s="56">
         <f>C22*(1-MIN(1,NB_LIGNES*D$5))+C21*MIN(1,NB_LIGNES*D$5)</f>
         <v/>
       </c>
-      <c r="E22" s="40">
+      <c r="E22" s="56">
         <f>D22*(1-MIN(1,NB_LIGNES*E$5))+D21*MIN(1,NB_LIGNES*E$5)</f>
         <v/>
       </c>
-      <c r="F22" s="40">
+      <c r="F22" s="56">
         <f>E22*(1-MIN(1,NB_LIGNES*F$5))+E21*MIN(1,NB_LIGNES*F$5)</f>
         <v/>
       </c>
-      <c r="G22" s="40">
+      <c r="G22" s="56">
         <f>IF($A22=0,1-MIN(1,NB_LIGNES*B$6),IF($A22=1,MIN(1,NB_LIGNES*B$6),0))</f>
         <v/>
       </c>
-      <c r="H22" s="40">
+      <c r="H22" s="56">
         <f>G22*(1-MIN(1,NB_LIGNES*C$6))+G21*MIN(1,NB_LIGNES*C$6)</f>
         <v/>
       </c>
-      <c r="I22" s="40">
+      <c r="I22" s="56">
         <f>H22*(1-MIN(1,NB_LIGNES*D$6))+H21*MIN(1,NB_LIGNES*D$6)</f>
         <v/>
       </c>
-      <c r="J22" s="40">
+      <c r="J22" s="56">
         <f>I22*(1-MIN(1,NB_LIGNES*E$6))+I21*MIN(1,NB_LIGNES*E$6)</f>
         <v/>
       </c>
-      <c r="K22" s="40">
+      <c r="K22" s="56">
         <f>J22*(1-MIN(1,NB_LIGNES*F$6))+J21*MIN(1,NB_LIGNES*F$6)</f>
         <v/>
       </c>
@@ -8771,43 +9198,43 @@
       <c r="A23" s="39" t="n">
         <v>5</v>
       </c>
-      <c r="B23" s="40">
+      <c r="B23" s="56">
         <f>IF($A23=0,1-MIN(1,NB_LIGNES*B$5),IF($A23=1,MIN(1,NB_LIGNES*B$5),0))</f>
         <v/>
       </c>
-      <c r="C23" s="40">
+      <c r="C23" s="56">
         <f>B23*(1-MIN(1,NB_LIGNES*C$5))+B22*MIN(1,NB_LIGNES*C$5)</f>
         <v/>
       </c>
-      <c r="D23" s="40">
+      <c r="D23" s="56">
         <f>C23*(1-MIN(1,NB_LIGNES*D$5))+C22*MIN(1,NB_LIGNES*D$5)</f>
         <v/>
       </c>
-      <c r="E23" s="40">
+      <c r="E23" s="56">
         <f>D23*(1-MIN(1,NB_LIGNES*E$5))+D22*MIN(1,NB_LIGNES*E$5)</f>
         <v/>
       </c>
-      <c r="F23" s="40">
+      <c r="F23" s="56">
         <f>E23*(1-MIN(1,NB_LIGNES*F$5))+E22*MIN(1,NB_LIGNES*F$5)</f>
         <v/>
       </c>
-      <c r="G23" s="40">
+      <c r="G23" s="56">
         <f>IF($A23=0,1-MIN(1,NB_LIGNES*B$6),IF($A23=1,MIN(1,NB_LIGNES*B$6),0))</f>
         <v/>
       </c>
-      <c r="H23" s="40">
+      <c r="H23" s="56">
         <f>G23*(1-MIN(1,NB_LIGNES*C$6))+G22*MIN(1,NB_LIGNES*C$6)</f>
         <v/>
       </c>
-      <c r="I23" s="40">
+      <c r="I23" s="56">
         <f>H23*(1-MIN(1,NB_LIGNES*D$6))+H22*MIN(1,NB_LIGNES*D$6)</f>
         <v/>
       </c>
-      <c r="J23" s="40">
+      <c r="J23" s="56">
         <f>I23*(1-MIN(1,NB_LIGNES*E$6))+I22*MIN(1,NB_LIGNES*E$6)</f>
         <v/>
       </c>
-      <c r="K23" s="40">
+      <c r="K23" s="56">
         <f>J23*(1-MIN(1,NB_LIGNES*F$6))+J22*MIN(1,NB_LIGNES*F$6)</f>
         <v/>
       </c>
@@ -8923,7 +9350,7 @@
           <t>base</t>
         </is>
       </c>
-      <c r="B34" s="36">
+      <c r="B34" s="53">
         <f>NB_LIGNES*SUM(B10:F10)</f>
         <v/>
       </c>
@@ -8938,7 +9365,7 @@
           <t>boost</t>
         </is>
       </c>
-      <c r="B35" s="36">
+      <c r="B35" s="53">
         <f>NB_LIGNES*SUM(B11:F11)</f>
         <v/>
       </c>
@@ -8953,7 +9380,7 @@
           <t>FS bonus 1</t>
         </is>
       </c>
-      <c r="B36" s="36">
+      <c r="B36" s="53">
         <f>NB_LIGNES*SUM(B12:F12)</f>
         <v/>
       </c>
@@ -8968,7 +9395,7 @@
           <t>FS bonus 2</t>
         </is>
       </c>
-      <c r="B37" s="36">
+      <c r="B37" s="53">
         <f>NB_LIGNES*SUM(B13:F13)</f>
         <v/>
       </c>
@@ -8983,7 +9410,7 @@
           <t>FS bonus 3</t>
         </is>
       </c>
-      <c r="B38" s="36">
+      <c r="B38" s="53">
         <f>NB_LIGNES*SUM(B14:F14)</f>
         <v/>
       </c>
@@ -9021,7 +9448,7 @@
         <f>Config!A25</f>
         <v/>
       </c>
-      <c r="B42" s="36">
+      <c r="B42" s="53">
         <f>NB_LIGNES*SUM(B7:F7)</f>
         <v/>
       </c>
@@ -9035,7 +9462,7 @@
         <f>Config!A26</f>
         <v/>
       </c>
-      <c r="B43" s="36">
+      <c r="B43" s="53">
         <f>NB_LIGNES*SUM(B8:F8)</f>
         <v/>
       </c>
@@ -9049,7 +9476,7 @@
         <f>Config!A27</f>
         <v/>
       </c>
-      <c r="B44" s="36">
+      <c r="B44" s="53">
         <f>NB_LIGNES*SUM(B9:F9)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Spins boostés à 1,25x (limite 3 étoiles respectée sans déformation), bonus 1 à 59x dans la spec
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014K11WNgkEUnnGsVcri14bC
</commit_message>
<xml_diff>
--- a/modele_maths/modele_maths.xlsx
+++ b/modele_maths/modele_maths.xlsx
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="B16" s="24" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
@@ -5458,19 +5458,19 @@
         <v/>
       </c>
       <c r="C26" s="19" t="n">
-        <v>1250</v>
+        <v>1135</v>
       </c>
       <c r="D26" s="19" t="n">
-        <v>1250</v>
+        <v>1135</v>
       </c>
       <c r="E26" s="19" t="n">
-        <v>1250</v>
+        <v>1135</v>
       </c>
       <c r="F26" s="19" t="n">
-        <v>1250</v>
+        <v>1135</v>
       </c>
       <c r="G26" s="19" t="n">
-        <v>1250</v>
+        <v>1135</v>
       </c>
       <c r="I26" s="29">
         <f>IF(C$28=0,0,C26/C$28)</f>

</xml_diff>

<commit_message>
Simulation des spins boostés à 1,25x et réexport SDK
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014K11WNgkEUnnGsVcri14bC
</commit_message>
<xml_diff>
--- a/modele_maths/modele_maths.xlsx
+++ b/modele_maths/modele_maths.xlsx
@@ -897,7 +897,7 @@
         <v>0.6996192733293443</v>
       </c>
       <c r="H5" s="56" t="n">
-        <v>0.7006786108775992</v>
+        <v>0.7007892950740482</v>
       </c>
     </row>
     <row r="6">
@@ -910,7 +910,7 @@
         <v>3078340</v>
       </c>
       <c r="C6" s="20" t="n">
-        <v>1532014</v>
+        <v>1535082</v>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         <v>0.180270346466384</v>
       </c>
       <c r="H6" s="56" t="n">
-        <v>0.1776766631435479</v>
+        <v>0.1784255975275916</v>
       </c>
     </row>
     <row r="7">
@@ -934,7 +934,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="44" t="n">
-        <v>1.5</v>
+        <v>1.25</v>
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
         <v>0.1107845617342869</v>
       </c>
       <c r="H7" s="56" t="n">
-        <v>0.1076111619620006</v>
+        <v>0.1089191759007165</v>
       </c>
     </row>
     <row r="8">
@@ -958,7 +958,7 @@
         <v>0.5888030533550216</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>0.371916280648126</v>
+        <v>0.4645806141650528</v>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
         <v>0.007767980995735308</v>
       </c>
       <c r="H8" s="56" t="n">
-        <v>0.01159278730710878</v>
+        <v>0.009833971923809415</v>
       </c>
     </row>
     <row r="9">
@@ -982,7 +982,7 @@
         <v>0.3568642256532524</v>
       </c>
       <c r="C9" s="29" t="n">
-        <v>0.5845663256446606</v>
+        <v>0.5197012661056304</v>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
@@ -993,7 +993,7 @@
         <v>0.0005480605065355157</v>
       </c>
       <c r="H9" s="56" t="n">
-        <v>0.0008497950419780626</v>
+        <v>0.0007293080700855172</v>
       </c>
     </row>
     <row r="10">
@@ -1006,7 +1006,7 @@
         <v>0.9456672790082743</v>
       </c>
       <c r="C10" s="29" t="n">
-        <v>0.9564826062927866</v>
+        <v>0.984281880270683</v>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
@@ -1017,7 +1017,7 @@
         <v>0.0008623815027859917</v>
       </c>
       <c r="H10" s="56" t="n">
-        <v>0.001276657364401604</v>
+        <v>0.001063976091671122</v>
       </c>
     </row>
     <row r="11">
@@ -1030,7 +1030,7 @@
         <v>0.0221287599106688</v>
       </c>
       <c r="C11" s="57" t="n">
-        <v>0.03274423528656293</v>
+        <v>0.03595189340215042</v>
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
@@ -1041,7 +1041,7 @@
         <v>0.0001473750433704121</v>
       </c>
       <c r="H11" s="56" t="n">
-        <v>0.0003142633685055289</v>
+        <v>0.0002386543380734879</v>
       </c>
     </row>
     <row r="12">
@@ -1054,7 +1054,7 @@
         <v>0.3003807266706552</v>
       </c>
       <c r="C12" s="29" t="n">
-        <v>0.2993213891224005</v>
+        <v>0.2992107049259518</v>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         <v>2.042155708400434e-08</v>
       </c>
       <c r="H12" s="56" t="n">
-        <v>6.093485803643417e-08</v>
+        <v>2.107400403580947e-08</v>
       </c>
     </row>
     <row r="13">
@@ -1078,7 +1078,7 @@
         <v>24.62485937985256</v>
       </c>
       <c r="C13" s="44" t="n">
-        <v>35.56933001456112</v>
+        <v>33.3147253852575</v>
       </c>
       <c r="F13" s="6" t="n"/>
       <c r="G13" s="57" t="n"/>
@@ -1094,7 +1094,7 @@
         <v>180.8611204466233</v>
       </c>
       <c r="C14" s="20" t="n">
-        <v>82.76905512847853</v>
+        <v>108.1091298326653</v>
       </c>
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="57" t="n"/>
@@ -1110,7 +1110,7 @@
         <v>191.617590769405</v>
       </c>
       <c r="C15" s="20" t="n">
-        <v>89.35743087087256</v>
+        <v>116.0726822694018</v>
       </c>
     </row>
     <row r="16">
@@ -1123,7 +1123,7 @@
         <v>3344.713124725586</v>
       </c>
       <c r="C16" s="20" t="n">
-        <v>1182.807573562243</v>
+        <v>1657.912134993445</v>
       </c>
     </row>
     <row r="17">
@@ -1136,7 +1136,7 @@
         <v>87738.89687603264</v>
       </c>
       <c r="C17" s="20" t="n">
-        <v>22049.31854210523</v>
+        <v>31793.72715816259</v>
       </c>
     </row>
     <row r="18">
@@ -1149,7 +1149,7 @@
         <v>56.03337221951441</v>
       </c>
       <c r="C18" s="51" t="n">
-        <v>60.66633288506777</v>
+        <v>58.08607784383116</v>
       </c>
     </row>
     <row r="19">
@@ -1162,7 +1162,7 @@
         <v>151.4935473851667</v>
       </c>
       <c r="C19" s="51" t="n">
-        <v>144.9355597016774</v>
+        <v>146.4051814212355</v>
       </c>
     </row>
     <row r="20">
@@ -1175,7 +1175,7 @@
         <v>1680.014489336063</v>
       </c>
       <c r="C20" s="51" t="n">
-        <v>1662.445562038904</v>
+        <v>1935.95584255784</v>
       </c>
     </row>
     <row r="21">
@@ -1188,7 +1188,7 @@
         <v>25.93482716889917</v>
       </c>
       <c r="C21" s="44" t="n">
-        <v>25.8400013258818</v>
+        <v>25.79774950362885</v>
       </c>
     </row>
     <row r="22">
@@ -1201,7 +1201,7 @@
         <v>30.79813034088118</v>
       </c>
       <c r="C22" s="44" t="n">
-        <v>31.06264515918089</v>
+        <v>30.83042691153424</v>
       </c>
     </row>
     <row r="23">
@@ -1214,7 +1214,7 @@
         <v>7.049432521777755</v>
       </c>
       <c r="C23" s="44" t="n">
-        <v>6.837250932294474</v>
+        <v>7.034164367770796</v>
       </c>
     </row>
     <row r="24">
@@ -1240,7 +1240,7 @@
         <v>0.0008836304957335275</v>
       </c>
       <c r="C25" s="29" t="n">
-        <v>0.0008619543919122412</v>
+        <v>0.0008771567291051974</v>
       </c>
     </row>
     <row r="26">
@@ -1253,7 +1253,7 @@
         <v>0.5812887374764568</v>
       </c>
       <c r="C26" s="58" t="n">
-        <v>1.026708547209999</v>
+        <v>0.8428394216561748</v>
       </c>
     </row>
     <row r="27">
@@ -1266,7 +1266,7 @@
         <v>0.0002042155708400434</v>
       </c>
       <c r="C27" s="58" t="n">
-        <v>0.0006093485803643417</v>
+        <v>0.0002107400403580947</v>
       </c>
     </row>
     <row r="28">
@@ -1279,7 +1279,7 @@
         <v>48967862.53303246</v>
       </c>
       <c r="C28" s="20" t="n">
-        <v>16410967.91268604</v>
+        <v>47451827.29873143</v>
       </c>
     </row>
     <row r="29">
@@ -1292,7 +1292,7 @@
         <v>0.005218727549932577</v>
       </c>
       <c r="C29" s="46" t="n">
-        <v>0.01119101109168041</v>
+        <v>0.0086152915608431</v>
       </c>
     </row>
     <row r="30">
@@ -1305,7 +1305,7 @@
         <v>0.0001480537857394944</v>
       </c>
       <c r="C30" s="46" t="n">
-        <v>0.0003972701767700076</v>
+        <v>0.0002932750441061707</v>
       </c>
     </row>
     <row r="31">
@@ -1318,7 +1318,7 @@
         <v>6.646147203031276e-06</v>
       </c>
       <c r="C31" s="46" t="n">
-        <v>2.631653734865039e-05</v>
+        <v>1.888146469125243e-05</v>
       </c>
     </row>
     <row r="32">
@@ -1344,7 +1344,7 @@
         <v>0.0001509255176293602</v>
       </c>
       <c r="C33" s="46" t="n">
-        <v>0.0004481758808580007</v>
+        <v>0.0003098932293466399</v>
       </c>
     </row>
     <row r="34">
@@ -1357,7 +1357,7 @@
         <v>2.236160500698488e-06</v>
       </c>
       <c r="C34" s="46" t="n">
-        <v>8.835554415283003e-06</v>
+        <v>6.216831190563829e-06</v>
       </c>
     </row>
     <row r="35">
@@ -1396,7 +1396,7 @@
         <v>2.515145827229671e-06</v>
       </c>
       <c r="C37" s="46" t="n">
-        <v>1.020078379507154e-05</v>
+        <v>6.354449341318956e-06</v>
       </c>
     </row>
     <row r="40">
@@ -2383,7 +2383,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
@@ -2649,8 +2648,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23">
       <c r="A23" s="12" t="inlineStr">
         <is>

</xml_diff>